<commit_message>
Restaurar cañería de acero LAP10AC en CAÑERIAS AP
El reemplazo de base_datos.xlsx por la versión de nota-de-venta-abastible
eliminó estas 15 filas (3 diámetros x 5 centros) porque el repo fuente no
las tenía. Se restauran con los mismos códigos y precios originales.
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="37.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2097,6 +2097,606 @@
       </c>
       <c r="H41" t="n">
         <v>8502</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LAP10AC 1" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1000099</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>16145</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>LAP10AC 1" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1000099</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>16145</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>LAP10AC 1" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1000099</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>16145</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>LAP10AC 1" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1000099</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>16145</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>LAP10AC 1" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1000099</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>16145</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LAP10AC 3/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1000104</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>13173</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>LAP10AC 3/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1000104</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>13173</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>LAP10AC 3/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1000104</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>13173</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>LAP10AC 3/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1000104</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>13173</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>LAP10AC 3/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1000104</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>13173</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>LAP10AC 1 1/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1000098</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>18826</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>LAP10AC 1 1/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1000098</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Arica</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>0300</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>18826</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>LAP10AC 1 1/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1000098</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Planta Iquique</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>0400</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>18826</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>LAP10AC 1 1/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>1000098</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Planta Antofagasta</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>0500</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>18826</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>LAP10AC 1 1/4" (Acero - Alta Presión, material incluido)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>1000098</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>CAÑERIAS AP</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>1 1/4</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Calama</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>0600</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>18826</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualiza precios Copiapo desde detalle comercial
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -1,31 +1,29 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="CAÑERIAS AP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="CAÑERIAS MP" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CAÑERIAS BP" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="SERVICIO CAÑERIAS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CONEXIONES" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="OBRAS CIVILES" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="NORMALIZACIONES" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="EQUIPO COMPRA DIRECTA" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="SERVICIO COMPRA DIRECTA" sheetId="9" state="visible" r:id="rId9"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CAÑERIAS AP'!$A$1:$G$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CAÑERIAS MP'!$A$1:$G$86</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CAÑERIAS BP'!$A$1:$H$86</definedName>
-  </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
+  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
+  <AppVersion>3.1</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>openpyxl</dc:creator>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-06-30T21:56:42Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-07-23T22:56:37Z</dcterms:modified>
+  <cp:lastModifiedBy>Daniel Villalobos Carrizo</cp:lastModifiedBy>
+</cp:coreProperties>
+</file>
+
+<file path=docProps\custom.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes" xmlns="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties">
+  <property name="KriptosClassAi" fmtid="{D5CDD505-2E9C-101B-9397-08002B2CF9AE}" pid="2">
+    <vt:lpwstr>1-Uso Interno</vt:lpwstr>
+  </property>
+</Properties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="1">
@@ -155,7 +153,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -438,7 +436,33 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="CAÑERIAS AP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CAÑERIAS MP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CAÑERIAS BP" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SERVICIO CAÑERIAS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CONEXIONES" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="OBRAS CIVILES" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="NORMALIZACIONES" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="EQUIPO COMPRA DIRECTA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SERVICIO COMPRA DIRECTA" sheetId="9" state="visible" r:id="rId9"/>
+  </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'CAÑERIAS AP'!$A$1:$G$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CAÑERIAS MP'!$A$1:$G$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'CAÑERIAS BP'!$A$1:$H$86</definedName>
+  </definedNames>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2117,7 +2141,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5213,7 +5237,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="78" hidden="1">
@@ -5588,7 +5612,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="1">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8685,7 +8709,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="78" hidden="1">
@@ -9060,7 +9084,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9141,7 +9165,7 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>3248</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="3">
@@ -9176,7 +9200,7 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>16238</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="4">
@@ -10689,13 +10713,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G271"/>
+  <dimension ref="A1:G273"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="12.5703125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -10840,7 +10864,7 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>29769</v>
+        <v>12784</v>
       </c>
     </row>
     <row r="5">
@@ -13745,7 +13769,7 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>54125</v>
+        <v>30899</v>
       </c>
     </row>
     <row r="88">
@@ -18435,7 +18459,7 @@
         </is>
       </c>
       <c r="G221" t="n">
-        <v>45248</v>
+        <v>31586</v>
       </c>
     </row>
     <row r="222">
@@ -18715,7 +18739,7 @@
         </is>
       </c>
       <c r="G229" t="n">
-        <v>70230</v>
+        <v>64878</v>
       </c>
     </row>
     <row r="230">
@@ -20186,6 +20210,76 @@
       </c>
       <c r="G271" t="n">
         <v>38000</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>CONEXIÓN VALV CORTE 1 1/2" ALTA PRESION</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1000241</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G271">
+        <v>94425</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>1000274</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G271">
+        <v>2500</v>
       </c>
     </row>
   </sheetData>
@@ -20193,13 +20287,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G126"/>
+  <dimension ref="A1:G127"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="14.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
@@ -20414,7 +20508,7 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>41175</v>
+        <v>30183</v>
       </c>
     </row>
     <row r="7">
@@ -23249,7 +23343,7 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>15155</v>
+        <v>7588</v>
       </c>
     </row>
     <row r="88">
@@ -23809,7 +23903,7 @@
         </is>
       </c>
       <c r="G103" t="n">
-        <v>108250</v>
+        <v>12271</v>
       </c>
     </row>
     <row r="104">
@@ -24299,7 +24393,7 @@
         </is>
       </c>
       <c r="G117" t="n">
-        <v>3789</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="118">
@@ -24615,6 +24709,41 @@
       </c>
       <c r="G126" t="n">
         <v>200000</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>MANO OBRA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1000690</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G126">
+        <v>20000</v>
       </c>
     </row>
   </sheetData>
@@ -24622,7 +24751,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25858,7 +25987,7 @@
         </is>
       </c>
       <c r="G35" t="n">
-        <v>16238</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="36">
@@ -28343,7 +28472,7 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>70362</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="107">
@@ -30618,7 +30747,7 @@
         </is>
       </c>
       <c r="G171" t="n">
-        <v>129900</v>
+        <v>105000</v>
       </c>
     </row>
   </sheetData>
@@ -30626,13 +30755,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G376"/>
+  <dimension ref="A1:G377"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="46.140625" customWidth="1" min="3" max="3"/>
@@ -41522,7 +41651,7 @@
         </is>
       </c>
       <c r="G311" t="n">
-        <v>35820</v>
+        <v>29536</v>
       </c>
     </row>
     <row r="312">
@@ -42047,7 +42176,7 @@
         </is>
       </c>
       <c r="G326" t="n">
-        <v>5644</v>
+        <v>5400</v>
       </c>
     </row>
     <row r="327">
@@ -42152,7 +42281,7 @@
         </is>
       </c>
       <c r="G329" t="n">
-        <v>8738</v>
+        <v>8006</v>
       </c>
     </row>
     <row r="330">
@@ -43798,6 +43927,41 @@
       </c>
       <c r="G376" t="n">
         <v>654371</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>REGULADOR 67/684 FISHER</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>000000000000004769</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>EQUIPO COMPRA DIRECTA</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Oficina Ventas Copiapó</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>0005</t>
+        </is>
+      </c>
+      <c r="G376">
+        <v>39579</v>
       </c>
     </row>
   </sheetData>
@@ -43805,7 +43969,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Trasladar MOI de Normalizaciones a Obras Civiles y agregar vigencia de cotización
Normalizaciones no puede llevar Mano de Obra Industrial propia: su diferencia
Renova/Contratista ahora se suma al MOI de Obras Civiles, como si fuera un
ítem libre de esa categoría (aplica igual en la vista web y en el Excel
exportado). También se elimina "MANO DE OBRA MANTENCION INDUSTRIAL" de la
base de datos (Conexiones), ya que el contratista no debe poder agregar MOI
como ítem de catálogo.

Se agrega además el campo "Vigencia de la cotización" (15/30/45 días) en
Datos del proyecto, que calcula y muestra la fecha "Válida hasta" a partir
de la Fecha, e incluye ambos datos en la cotización guardada/cargada y en
el Excel exportado.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PcPgm3zC8vk1tLVWURq5kH
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -20247,41 +20247,6 @@
         <v>94425</v>
       </c>
     </row>
-    <row r="273">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t>MANO DE OBRA MANTENCION INDUSTRIAL</t>
-        </is>
-      </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t>1000274</t>
-        </is>
-      </c>
-      <c r="C271" t="inlineStr">
-        <is>
-          <t>CONEXIONES</t>
-        </is>
-      </c>
-      <c r="D271" t="inlineStr">
-        <is>
-          <t>ST</t>
-        </is>
-      </c>
-      <c r="E271" t="inlineStr">
-        <is>
-          <t>Oficina Ventas Copiapó</t>
-        </is>
-      </c>
-      <c r="F271" t="inlineStr">
-        <is>
-          <t>0005</t>
-        </is>
-      </c>
-      <c r="G271">
-        <v>2500</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Agregar items faltantes de San Fernando a base de datos
Se analizaron 5 Detalle Comercial (SOLPED) de proyectos VI Región
(Rancagua) y se identificaron ítems de servicios/conexiones/obras
civiles/normalizaciones que ya existen en el catálogo para otros
centros pero faltaban para "Oficina Ventas San Fernando" (0110),
además de 10 códigos nuevos que no existían para ningún centro.
Se agregaron usando el precio consistente observado en los 5 DC.

- SERVICIO CAÑERIAS: 4 ítems
- CONEXIONES: 17 ítems
- OBRAS CIVILES: 9 ítems
- NORMALIZACIONES: 3 ítems

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NXmK2PLE7T5P6GP4FqzB9A
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -22429,7 +22429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24182,6 +24182,146 @@
       </c>
       <c r="G50" t="n">
         <v>4800</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DETECCION ESCAPE</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1000046</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>VIATICO TRASLADO</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1000640</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>MANO OBRA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1000690</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ANCLAJE Y PINTURA CAÑERIA AEREA</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1001200</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>3000</v>
       </c>
     </row>
   </sheetData>
@@ -24195,7 +24335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G250"/>
+  <dimension ref="A1:G267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32948,6 +33088,601 @@
       </c>
       <c r="G250" t="n">
         <v>20000</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>CONEXIÓN ANAFE INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>1000005</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G251" t="n">
+        <v>9744</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FLEXIBLES 3/4"</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>1000058</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G252" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>GABINETE PROTECCION CALEFON</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>1000069</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G253" t="n">
+        <v>23750</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>CONEXIÓN HORNO INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>1000075</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G254" t="n">
+        <v>320000</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>INTERCONEXION SERV. P/ 3 EST. AEREOS DE</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>1000087</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G255" t="n">
+        <v>134565</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>VENTILACION CALEFONT 5"</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>1000267</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G256" t="n">
+        <v>20726</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>VIATICO TRASLADO</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>1000640</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G257" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>VIATICO ALIMENTACION</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>1000642</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G258" t="n">
+        <v>2752</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>MANO OBRA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>1000690</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G259" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>MANIFOLD INTERCONEXION 2 S.BALON AEREOS</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1001700</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>64878</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>MANIFOLD INTERCONEXION 3 S.BALON AEREOS</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1001701</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G261" t="n">
+        <v>107028</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 3/4"</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>1000190</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G262" t="n">
+        <v>28597</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>CONEXIÓN HORNO DOMESTICO</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>1000074</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G263" t="n">
+        <v>11990</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR ETAPA UNICA</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>1000630</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G264" t="n">
+        <v>26419</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>CONEXION HORNO DOM-COM 3/4"</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>1001213</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G265" t="n">
+        <v>19995</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>CONEXIÓN ESTUFA MURAL</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>1000054</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G266" t="n">
+        <v>11792</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>CONEXIÓN AGUA CALEFONT</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>1000004</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G267" t="n">
+        <v>13480</v>
       </c>
     </row>
   </sheetData>
@@ -32961,7 +33696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G226"/>
+  <dimension ref="A1:G235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40874,6 +41609,321 @@
       </c>
       <c r="G226" t="n">
         <v>20000</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>ANCLAJE DE ESTANQUE AEREO HASTA 4000 LTS</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>1000006</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G227" t="n">
+        <v>7588</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>BASES ESTANQUE SUPER BALON 190 KG.</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>1000013</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G228" t="n">
+        <v>12271</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>PROTECCION METALICA PARA REGULADOR</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G229" t="n">
+        <v>8500</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>MANO OBRA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1000690</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G230" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>CELOSIA EN MURO CON TESTIGUERA</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>1000962</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G231" t="n">
+        <v>28261</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>REJA ESTANQUE SUPERBALON 190</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>1000219</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G232" t="n">
+        <v>200417</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>VENTILACION 5 1/2" DOBLE</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1000265</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G233" t="n">
+        <v>21373</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>INSTALACION CODO 45 P/ VENTILACION DE 5"</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1000851</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G234" t="n">
+        <v>6769</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>BASE DE CEMENTO 2 X 45 KGS.</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>1000010</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G235" t="n">
+        <v>13000</v>
       </c>
     </row>
   </sheetData>
@@ -40887,7 +41937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G430"/>
+  <dimension ref="A1:G433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55940,6 +56990,111 @@
       </c>
       <c r="G430" t="n">
         <v>50000</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>MANO OBRA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>1000690</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G431" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>CERTIFICACION INTEGRAL COMERCIAL</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>1000819</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G432" t="n">
+        <v>117414</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>1001879</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G433" t="n">
+        <v>60000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregar items faltantes de San Fernando a base de datos (#17)
Se analizaron 5 Detalle Comercial (SOLPED) de proyectos VI Región
(Rancagua) y se identificaron ítems de servicios/conexiones/obras
civiles/normalizaciones que ya existen en el catálogo para otros
centros pero faltaban para "Oficina Ventas San Fernando" (0110),
además de 10 códigos nuevos que no existían para ningún centro.
Se agregaron usando el precio consistente observado en los 5 DC.

- SERVICIO CAÑERIAS: 4 ítems
- CONEXIONES: 17 ítems
- OBRAS CIVILES: 9 ítems
- NORMALIZACIONES: 3 ítems


Claude-Session: https://claude.ai/code/session_01NXmK2PLE7T5P6GP4FqzB9A

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -22429,7 +22429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24182,6 +24182,146 @@
       </c>
       <c r="G50" t="n">
         <v>4800</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DETECCION ESCAPE</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1000046</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>7500</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>VIATICO TRASLADO</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1000640</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>MANO OBRA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>1000690</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ANCLAJE Y PINTURA CAÑERIA AEREA</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1001200</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SERVICIO CAÑERIAS</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>3000</v>
       </c>
     </row>
   </sheetData>
@@ -24195,7 +24335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G250"/>
+  <dimension ref="A1:G267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32948,6 +33088,601 @@
       </c>
       <c r="G250" t="n">
         <v>20000</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>CONEXIÓN ANAFE INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>1000005</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G251" t="n">
+        <v>9744</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>CONEXIÓN FLEXIBLES 3/4"</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>1000058</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G252" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>GABINETE PROTECCION CALEFON</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>1000069</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G253" t="n">
+        <v>23750</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>CONEXIÓN HORNO INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>1000075</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G254" t="n">
+        <v>320000</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>INTERCONEXION SERV. P/ 3 EST. AEREOS DE</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>1000087</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G255" t="n">
+        <v>134565</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>VENTILACION CALEFONT 5"</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>1000267</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G256" t="n">
+        <v>20726</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>VIATICO TRASLADO</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>1000640</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>KM</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G257" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>VIATICO ALIMENTACION</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>1000642</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G258" t="n">
+        <v>2752</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>MANO OBRA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>1000690</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G259" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>MANIFOLD INTERCONEXION 2 S.BALON AEREOS</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>1001700</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>64878</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>MANIFOLD INTERCONEXION 3 S.BALON AEREOS</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>1001701</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G261" t="n">
+        <v>107028</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>CONEXIÓN QUEMADOR INDUSTRIAL,RED EN 3/4"</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>1000190</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G262" t="n">
+        <v>28597</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>CONEXIÓN HORNO DOMESTICO</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>1000074</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G263" t="n">
+        <v>11990</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>CONEXIÓN REGULADOR ETAPA UNICA</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>1000630</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G264" t="n">
+        <v>26419</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>CONEXION HORNO DOM-COM 3/4"</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>1001213</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G265" t="n">
+        <v>19995</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>CONEXIÓN ESTUFA MURAL</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>1000054</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G266" t="n">
+        <v>11792</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>CONEXIÓN AGUA CALEFONT</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>1000004</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>CONEXIONES</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G267" t="n">
+        <v>13480</v>
       </c>
     </row>
   </sheetData>
@@ -32961,7 +33696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G226"/>
+  <dimension ref="A1:G235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40874,6 +41609,321 @@
       </c>
       <c r="G226" t="n">
         <v>20000</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>ANCLAJE DE ESTANQUE AEREO HASTA 4000 LTS</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>1000006</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G227" t="n">
+        <v>7588</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>BASES ESTANQUE SUPER BALON 190 KG.</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>1000013</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G228" t="n">
+        <v>12271</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>PROTECCION METALICA PARA REGULADOR</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>1000181</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G229" t="n">
+        <v>8500</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>MANO OBRA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>1000690</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G230" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>CELOSIA EN MURO CON TESTIGUERA</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>1000962</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G231" t="n">
+        <v>28261</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>REJA ESTANQUE SUPERBALON 190</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>1000219</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G232" t="n">
+        <v>200417</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>VENTILACION 5 1/2" DOBLE</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>1000265</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G233" t="n">
+        <v>21373</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>INSTALACION CODO 45 P/ VENTILACION DE 5"</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>1000851</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G234" t="n">
+        <v>6769</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>BASE DE CEMENTO 2 X 45 KGS.</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>1000010</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>OBRAS CIVILES</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G235" t="n">
+        <v>13000</v>
       </c>
     </row>
   </sheetData>
@@ -40887,7 +41937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G430"/>
+  <dimension ref="A1:G433"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55940,6 +56990,111 @@
       </c>
       <c r="G430" t="n">
         <v>50000</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>MANO OBRA INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>1000690</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G431" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>CERTIFICACION INTEGRAL COMERCIAL</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>1000819</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G432" t="n">
+        <v>117414</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>VISITAS REGULARI. DE INSTALACI. GRANEL</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>1001879</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>NORMALIZACIONES</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>ST</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Oficina Ventas San Fernando</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>0110</t>
+        </is>
+      </c>
+      <c r="G433" t="n">
+        <v>60000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Unificar precios de instalacion de canerias en los 13 centros
Se actualiza el precio de instalacion de canerias Cu (Alta, Media y
Baja Presion) para que sea el mismo en los 13 centros y coincida entre
las 3 categorias (AP/MP/BP) para un mismo diametro, usando la tarifa
vigente confirmada por Detalles Comerciales de 3 regiones distintas
(VI Rancagua, XV Arica, I Iquique): 3/8"=$9.382, 1/2"=$9.382,
3/4"=$9.382, 1"=$10.125, 1 1/4=$10.546, 1 1/2=$10.942, y 3"=$12.928
(diametro nuevo, sin precio previo confirmado).

Los diametros sin evidencia en los DC (2", 2 1/2", 4") y los items de
canerias protegida/rollo quedan sin cambios.
</commit_message>
<xml_diff>
--- a/base_datos.xlsx
+++ b/base_datos.xlsx
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="3">
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="4">
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="5">
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="6">
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="7">
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="8">
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="9">
@@ -794,7 +794,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="10">
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="11">
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="12">
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="13">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="14">
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="15">
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="16">
@@ -1074,7 +1074,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="17">
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="18">
@@ -1154,7 +1154,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="19">
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="20">
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="21">
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="22">
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="23">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="24">
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="25">
@@ -1434,7 +1434,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="26">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="27">
@@ -1514,7 +1514,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="28">
@@ -1554,7 +1554,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="29">
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="30">
@@ -1634,7 +1634,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="31">
@@ -1674,7 +1674,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="32">
@@ -1714,7 +1714,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="33">
@@ -1754,7 +1754,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="34">
@@ -1794,7 +1794,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="35">
@@ -1834,7 +1834,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="36">
@@ -1874,7 +1874,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="37">
@@ -1914,7 +1914,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="38">
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="39">
@@ -1994,7 +1994,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="40">
@@ -2034,7 +2034,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="41">
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="42">
@@ -2114,7 +2114,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="43">
@@ -2154,7 +2154,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="44">
@@ -2194,7 +2194,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="45">
@@ -2234,7 +2234,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="46">
@@ -2274,7 +2274,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="47">
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="48">
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="49">
@@ -2394,7 +2394,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="50">
@@ -2434,7 +2434,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="51">
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="52">
@@ -2514,7 +2514,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="53">
@@ -2554,7 +2554,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="54">
@@ -3634,7 +3634,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="81">
@@ -3674,7 +3674,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="82">
@@ -3714,7 +3714,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="83">
@@ -3754,7 +3754,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="84">
@@ -3794,7 +3794,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="85">
@@ -3834,7 +3834,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="86">
@@ -3874,7 +3874,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="87">
@@ -3914,7 +3914,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="88">
@@ -3954,7 +3954,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="89">
@@ -3994,7 +3994,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="90">
@@ -4034,7 +4034,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="91">
@@ -4074,7 +4074,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="92">
@@ -4114,7 +4114,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="93">
@@ -4154,7 +4154,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="94">
@@ -4194,7 +4194,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="95">
@@ -4234,7 +4234,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="96">
@@ -4274,7 +4274,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="97">
@@ -4314,7 +4314,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="98">
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="99">
@@ -4394,7 +4394,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="100">
@@ -4434,7 +4434,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="101">
@@ -4474,7 +4474,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="102">
@@ -4514,7 +4514,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="103">
@@ -4554,7 +4554,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="104">
@@ -4594,7 +4594,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="105">
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
   </sheetData>
@@ -8370,7 +8370,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="94">
@@ -8410,7 +8410,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="95">
@@ -8450,7 +8450,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="96">
@@ -8490,7 +8490,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="97">
@@ -8570,7 +8570,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="99">
@@ -8610,7 +8610,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="100">
@@ -8650,7 +8650,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="101">
@@ -8690,7 +8690,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="102">
@@ -8730,7 +8730,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="103">
@@ -8770,7 +8770,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="104">
@@ -8810,7 +8810,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="105">
@@ -8850,7 +8850,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="106">
@@ -8890,7 +8890,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="107">
@@ -8930,7 +8930,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="108">
@@ -8970,7 +8970,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="109">
@@ -9010,7 +9010,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="110">
@@ -9090,7 +9090,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="112">
@@ -9130,7 +9130,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="113">
@@ -9170,7 +9170,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="114">
@@ -9210,7 +9210,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="115">
@@ -9250,7 +9250,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="116">
@@ -9290,7 +9290,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="117">
@@ -9330,7 +9330,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="118">
@@ -9370,7 +9370,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="119">
@@ -9410,7 +9410,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="120">
@@ -9450,7 +9450,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="121">
@@ -9490,7 +9490,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="122">
@@ -9530,7 +9530,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="123">
@@ -9610,7 +9610,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="125">
@@ -9650,7 +9650,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="126">
@@ -9690,7 +9690,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="127">
@@ -9730,7 +9730,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="128">
@@ -9770,7 +9770,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="129">
@@ -9810,7 +9810,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="130">
@@ -9850,7 +9850,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="131">
@@ -9890,7 +9890,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="132">
@@ -9930,7 +9930,7 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="133">
@@ -9970,7 +9970,7 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="134">
@@ -10010,7 +10010,7 @@
         </is>
       </c>
       <c r="H134" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="135">
@@ -10050,7 +10050,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="136">
@@ -10130,7 +10130,7 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="138">
@@ -10170,7 +10170,7 @@
         </is>
       </c>
       <c r="H138" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="139">
@@ -10210,7 +10210,7 @@
         </is>
       </c>
       <c r="H139" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="140">
@@ -10250,7 +10250,7 @@
         </is>
       </c>
       <c r="H140" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="141">
@@ -10290,7 +10290,7 @@
         </is>
       </c>
       <c r="H141" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="142">
@@ -10330,7 +10330,7 @@
         </is>
       </c>
       <c r="H142" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="143">
@@ -10370,7 +10370,7 @@
         </is>
       </c>
       <c r="H143" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="144">
@@ -10410,7 +10410,7 @@
         </is>
       </c>
       <c r="H144" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="145">
@@ -11490,7 +11490,7 @@
         </is>
       </c>
       <c r="H171" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="172">
@@ -11530,7 +11530,7 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="173">
@@ -11570,7 +11570,7 @@
         </is>
       </c>
       <c r="H173" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="174">
@@ -11610,7 +11610,7 @@
         </is>
       </c>
       <c r="H174" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="175">
@@ -11650,7 +11650,7 @@
         </is>
       </c>
       <c r="H175" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="176">
@@ -11690,7 +11690,7 @@
         </is>
       </c>
       <c r="H176" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="177">
@@ -11730,7 +11730,7 @@
         </is>
       </c>
       <c r="H177" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="178">
@@ -11770,7 +11770,7 @@
         </is>
       </c>
       <c r="H178" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="179">
@@ -11810,7 +11810,7 @@
         </is>
       </c>
       <c r="H179" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="180">
@@ -11850,7 +11850,7 @@
         </is>
       </c>
       <c r="H180" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="181">
@@ -11890,7 +11890,7 @@
         </is>
       </c>
       <c r="H181" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="182">
@@ -11930,7 +11930,7 @@
         </is>
       </c>
       <c r="H182" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="183">
@@ -11970,7 +11970,7 @@
         </is>
       </c>
       <c r="H183" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="184">
@@ -12010,7 +12010,7 @@
         </is>
       </c>
       <c r="H184" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="185">
@@ -12050,7 +12050,7 @@
         </is>
       </c>
       <c r="H185" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="186">
@@ -12090,7 +12090,7 @@
         </is>
       </c>
       <c r="H186" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="187">
@@ -12130,7 +12130,7 @@
         </is>
       </c>
       <c r="H187" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="188">
@@ -12210,7 +12210,7 @@
         </is>
       </c>
       <c r="H189" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="190">
@@ -12250,7 +12250,7 @@
         </is>
       </c>
       <c r="H190" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="191">
@@ -12290,7 +12290,7 @@
         </is>
       </c>
       <c r="H191" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="192">
@@ -12330,7 +12330,7 @@
         </is>
       </c>
       <c r="H192" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="193">
@@ -12370,7 +12370,7 @@
         </is>
       </c>
       <c r="H193" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="194">
@@ -12410,7 +12410,7 @@
         </is>
       </c>
       <c r="H194" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="195">
@@ -12450,7 +12450,7 @@
         </is>
       </c>
       <c r="H195" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="196">
@@ -12490,7 +12490,7 @@
         </is>
       </c>
       <c r="H196" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="197">
@@ -12530,7 +12530,7 @@
         </is>
       </c>
       <c r="H197" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="198">
@@ -12570,7 +12570,7 @@
         </is>
       </c>
       <c r="H198" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="199">
@@ -12610,7 +12610,7 @@
         </is>
       </c>
       <c r="H199" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="200">
@@ -12650,7 +12650,7 @@
         </is>
       </c>
       <c r="H200" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="201">
@@ -12730,7 +12730,7 @@
         </is>
       </c>
       <c r="H202" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="203">
@@ -12770,7 +12770,7 @@
         </is>
       </c>
       <c r="H203" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="204">
@@ -12810,7 +12810,7 @@
         </is>
       </c>
       <c r="H204" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="205">
@@ -12850,7 +12850,7 @@
         </is>
       </c>
       <c r="H205" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="206">
@@ -12890,7 +12890,7 @@
         </is>
       </c>
       <c r="H206" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="207">
@@ -12930,7 +12930,7 @@
         </is>
       </c>
       <c r="H207" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="208">
@@ -12970,7 +12970,7 @@
         </is>
       </c>
       <c r="H208" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="209">
@@ -13010,7 +13010,7 @@
         </is>
       </c>
       <c r="H209" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="210">
@@ -17266,7 +17266,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="94">
@@ -17306,7 +17306,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="95">
@@ -17346,7 +17346,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="96">
@@ -17386,7 +17386,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="97">
@@ -17466,7 +17466,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="99">
@@ -17506,7 +17506,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="100">
@@ -17546,7 +17546,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="101">
@@ -17586,7 +17586,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="102">
@@ -17626,7 +17626,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="103">
@@ -17666,7 +17666,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="104">
@@ -17706,7 +17706,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="105">
@@ -17746,7 +17746,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>9916</v>
+        <v>10942</v>
       </c>
     </row>
     <row r="106">
@@ -17786,7 +17786,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="107">
@@ -17826,7 +17826,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="108">
@@ -17866,7 +17866,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="109">
@@ -17906,7 +17906,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="110">
@@ -17986,7 +17986,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="112">
@@ -18026,7 +18026,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="113">
@@ -18066,7 +18066,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="114">
@@ -18106,7 +18106,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="115">
@@ -18146,7 +18146,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="116">
@@ -18186,7 +18186,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="117">
@@ -18226,7 +18226,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="118">
@@ -18266,7 +18266,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>9557</v>
+        <v>10546</v>
       </c>
     </row>
     <row r="119">
@@ -18306,7 +18306,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="120">
@@ -18346,7 +18346,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="121">
@@ -18386,7 +18386,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="122">
@@ -18426,7 +18426,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="123">
@@ -18506,7 +18506,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="125">
@@ -18546,7 +18546,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="126">
@@ -18586,7 +18586,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="127">
@@ -18626,7 +18626,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="128">
@@ -18666,7 +18666,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="129">
@@ -18706,7 +18706,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="130">
@@ -18746,7 +18746,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="131">
@@ -18786,7 +18786,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>9175</v>
+        <v>10125</v>
       </c>
     </row>
     <row r="132">
@@ -18826,7 +18826,7 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="133">
@@ -18866,7 +18866,7 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="134">
@@ -18906,7 +18906,7 @@
         </is>
       </c>
       <c r="H134" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="135">
@@ -18946,7 +18946,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="136">
@@ -19026,7 +19026,7 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="138">
@@ -19066,7 +19066,7 @@
         </is>
       </c>
       <c r="H138" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="139">
@@ -19106,7 +19106,7 @@
         </is>
       </c>
       <c r="H139" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="140">
@@ -19146,7 +19146,7 @@
         </is>
       </c>
       <c r="H140" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="141">
@@ -19186,7 +19186,7 @@
         </is>
       </c>
       <c r="H141" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="142">
@@ -19226,7 +19226,7 @@
         </is>
       </c>
       <c r="H142" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="143">
@@ -19266,7 +19266,7 @@
         </is>
       </c>
       <c r="H143" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="144">
@@ -19306,7 +19306,7 @@
         </is>
       </c>
       <c r="H144" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="145">
@@ -20386,7 +20386,7 @@
         </is>
       </c>
       <c r="H171" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="172">
@@ -20426,7 +20426,7 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="173">
@@ -20466,7 +20466,7 @@
         </is>
       </c>
       <c r="H173" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="174">
@@ -20506,7 +20506,7 @@
         </is>
       </c>
       <c r="H174" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="175">
@@ -20546,7 +20546,7 @@
         </is>
       </c>
       <c r="H175" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="176">
@@ -20586,7 +20586,7 @@
         </is>
       </c>
       <c r="H176" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="177">
@@ -20626,7 +20626,7 @@
         </is>
       </c>
       <c r="H177" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="178">
@@ -20666,7 +20666,7 @@
         </is>
       </c>
       <c r="H178" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="179">
@@ -20706,7 +20706,7 @@
         </is>
       </c>
       <c r="H179" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="180">
@@ -20746,7 +20746,7 @@
         </is>
       </c>
       <c r="H180" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="181">
@@ -20786,7 +20786,7 @@
         </is>
       </c>
       <c r="H181" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="182">
@@ -20826,7 +20826,7 @@
         </is>
       </c>
       <c r="H182" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="183">
@@ -20866,7 +20866,7 @@
         </is>
       </c>
       <c r="H183" t="n">
-        <v>11715</v>
+        <v>12928</v>
       </c>
     </row>
     <row r="184">
@@ -20906,7 +20906,7 @@
         </is>
       </c>
       <c r="H184" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="185">
@@ -20946,7 +20946,7 @@
         </is>
       </c>
       <c r="H185" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="186">
@@ -20986,7 +20986,7 @@
         </is>
       </c>
       <c r="H186" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="187">
@@ -21026,7 +21026,7 @@
         </is>
       </c>
       <c r="H187" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="188">
@@ -21106,7 +21106,7 @@
         </is>
       </c>
       <c r="H189" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="190">
@@ -21146,7 +21146,7 @@
         </is>
       </c>
       <c r="H190" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="191">
@@ -21186,7 +21186,7 @@
         </is>
       </c>
       <c r="H191" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="192">
@@ -21226,7 +21226,7 @@
         </is>
       </c>
       <c r="H192" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="193">
@@ -21266,7 +21266,7 @@
         </is>
       </c>
       <c r="H193" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="194">
@@ -21306,7 +21306,7 @@
         </is>
       </c>
       <c r="H194" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="195">
@@ -21346,7 +21346,7 @@
         </is>
       </c>
       <c r="H195" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="196">
@@ -21386,7 +21386,7 @@
         </is>
       </c>
       <c r="H196" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="197">
@@ -21426,7 +21426,7 @@
         </is>
       </c>
       <c r="H197" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="198">
@@ -21466,7 +21466,7 @@
         </is>
       </c>
       <c r="H198" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="199">
@@ -21506,7 +21506,7 @@
         </is>
       </c>
       <c r="H199" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="200">
@@ -21546,7 +21546,7 @@
         </is>
       </c>
       <c r="H200" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="201">
@@ -21626,7 +21626,7 @@
         </is>
       </c>
       <c r="H202" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="203">
@@ -21666,7 +21666,7 @@
         </is>
       </c>
       <c r="H203" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="204">
@@ -21706,7 +21706,7 @@
         </is>
       </c>
       <c r="H204" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="205">
@@ -21746,7 +21746,7 @@
         </is>
       </c>
       <c r="H205" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="206">
@@ -21786,7 +21786,7 @@
         </is>
       </c>
       <c r="H206" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="207">
@@ -21826,7 +21826,7 @@
         </is>
       </c>
       <c r="H207" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="208">
@@ -21866,7 +21866,7 @@
         </is>
       </c>
       <c r="H208" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="209">
@@ -21906,7 +21906,7 @@
         </is>
       </c>
       <c r="H209" t="n">
-        <v>8502</v>
+        <v>9382</v>
       </c>
     </row>
     <row r="210">

</xml_diff>